<commit_message>
fix: update production excel templates
</commit_message>
<xml_diff>
--- a/app/templates/Template_Compresion.xlsx
+++ b/app/templates/Template_Compresion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC946D67-3543-4B91-A60C-9859211B861B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448594CE-AF0B-4DD2-9B69-10FFD032C8E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7452" yWindow="1788" windowWidth="16284" windowHeight="9828" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="92" r:id="rId1"/>
@@ -75,9 +75,6 @@
     <t>Página 1 de 1</t>
   </si>
   <si>
-    <t>Versión: 02 (09-09-2024)</t>
-  </si>
-  <si>
     <t>WEB: www.geofal.com.pe   E-MAIL: laboratorio@geofal.com.pe                                                                                                                                                                                 Av. Marañon 763, Los Olivos-Lima / Teléfono  01 754-3070</t>
   </si>
   <si>
@@ -103,6 +100,9 @@
   </si>
   <si>
     <t>Realizado</t>
+  </si>
+  <si>
+    <t>Versión: 04 (23-03-2026)</t>
   </si>
 </sst>
 </file>
@@ -641,6 +641,19 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="14" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -679,19 +692,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="14" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1682,44 +1682,44 @@
       <c r="N6" s="4"/>
     </row>
     <row r="7" spans="1:26" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="67" t="s">
+      <c r="A7" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="67"/>
-      <c r="C7" s="67"/>
-      <c r="D7" s="67"/>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="67"/>
-      <c r="H7" s="67"/>
-      <c r="I7" s="67"/>
-      <c r="J7" s="67"/>
-      <c r="K7" s="67"/>
-      <c r="L7" s="67"/>
-      <c r="M7" s="67"/>
-      <c r="N7" s="67"/>
+      <c r="B7" s="57"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="57"/>
+      <c r="E7" s="57"/>
+      <c r="F7" s="57"/>
+      <c r="G7" s="57"/>
+      <c r="H7" s="57"/>
+      <c r="I7" s="57"/>
+      <c r="J7" s="57"/>
+      <c r="K7" s="57"/>
+      <c r="L7" s="57"/>
+      <c r="M7" s="57"/>
+      <c r="N7" s="57"/>
     </row>
     <row r="8" spans="1:26" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="68" t="s">
+      <c r="A8" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="68"/>
-      <c r="C8" s="68"/>
-      <c r="D8" s="68"/>
-      <c r="E8" s="68"/>
-      <c r="F8" s="68"/>
-      <c r="G8" s="68"/>
-      <c r="H8" s="68"/>
-      <c r="I8" s="68"/>
-      <c r="J8" s="68"/>
-      <c r="K8" s="68"/>
-      <c r="L8" s="68"/>
-      <c r="M8" s="68"/>
-      <c r="N8" s="68"/>
-      <c r="V8" s="70"/>
-      <c r="W8" s="70"/>
-      <c r="X8" s="70"/>
-      <c r="Y8" s="70"/>
+      <c r="B8" s="58"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="58"/>
+      <c r="F8" s="58"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="58"/>
+      <c r="I8" s="58"/>
+      <c r="J8" s="58"/>
+      <c r="K8" s="58"/>
+      <c r="L8" s="58"/>
+      <c r="M8" s="58"/>
+      <c r="N8" s="58"/>
+      <c r="V8" s="60"/>
+      <c r="W8" s="60"/>
+      <c r="X8" s="60"/>
+      <c r="Y8" s="60"/>
       <c r="Z8" s="15"/>
     </row>
     <row r="9" spans="1:26" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -1735,10 +1735,10 @@
       <c r="L9" s="13"/>
       <c r="M9" s="13"/>
       <c r="N9" s="13"/>
-      <c r="V9" s="70"/>
-      <c r="W9" s="70"/>
-      <c r="X9" s="70"/>
-      <c r="Y9" s="70"/>
+      <c r="V9" s="60"/>
+      <c r="W9" s="60"/>
+      <c r="X9" s="60"/>
+      <c r="Y9" s="60"/>
       <c r="Z9" s="15"/>
     </row>
     <row r="10" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1762,47 +1762,47 @@
       <c r="N11" s="13"/>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
-      <c r="S11" s="60"/>
-      <c r="T11" s="60"/>
+      <c r="S11" s="64"/>
+      <c r="T11" s="64"/>
     </row>
     <row r="12" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="61" t="s">
+      <c r="A12" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
-      <c r="G12" s="62"/>
-      <c r="H12" s="62"/>
-      <c r="I12" s="62"/>
-      <c r="J12" s="62"/>
-      <c r="K12" s="62"/>
-      <c r="L12" s="62"/>
-      <c r="M12" s="62"/>
-      <c r="N12" s="63"/>
+      <c r="B12" s="66"/>
+      <c r="C12" s="66"/>
+      <c r="D12" s="66"/>
+      <c r="E12" s="66"/>
+      <c r="F12" s="66"/>
+      <c r="G12" s="66"/>
+      <c r="H12" s="66"/>
+      <c r="I12" s="66"/>
+      <c r="J12" s="66"/>
+      <c r="K12" s="66"/>
+      <c r="L12" s="66"/>
+      <c r="M12" s="66"/>
+      <c r="N12" s="67"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
     </row>
     <row r="13" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="64" t="s">
+      <c r="A13" s="68" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="65"/>
-      <c r="C13" s="65"/>
-      <c r="D13" s="65"/>
-      <c r="E13" s="65"/>
-      <c r="F13" s="65"/>
-      <c r="G13" s="65"/>
-      <c r="H13" s="65"/>
-      <c r="I13" s="65"/>
-      <c r="J13" s="65"/>
-      <c r="K13" s="65"/>
-      <c r="L13" s="65"/>
-      <c r="M13" s="65"/>
-      <c r="N13" s="66"/>
+      <c r="B13" s="69"/>
+      <c r="C13" s="69"/>
+      <c r="D13" s="69"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="69"/>
+      <c r="G13" s="69"/>
+      <c r="H13" s="69"/>
+      <c r="I13" s="69"/>
+      <c r="J13" s="69"/>
+      <c r="K13" s="69"/>
+      <c r="L13" s="69"/>
+      <c r="M13" s="69"/>
+      <c r="N13" s="70"/>
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
@@ -1813,13 +1813,13 @@
     </row>
     <row r="15" spans="1:26" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="41" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C15" s="41" t="s">
         <v>4</v>
       </c>
       <c r="D15" s="42" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E15" s="43" t="s">
         <v>5</v>
@@ -1831,22 +1831,22 @@
         <v>8</v>
       </c>
       <c r="H15" s="43" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I15" s="43" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J15" s="43" t="s">
         <v>7</v>
       </c>
       <c r="K15" s="43" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L15" s="43" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M15" s="43" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
@@ -2190,8 +2190,8 @@
       <c r="T33" s="20"/>
       <c r="U33" s="20"/>
       <c r="V33" s="20"/>
-      <c r="W33" s="69"/>
-      <c r="X33" s="69"/>
+      <c r="W33" s="59"/>
+      <c r="X33" s="59"/>
     </row>
     <row r="34" spans="1:27" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="35"/>
@@ -2219,18 +2219,18 @@
     <row r="35" spans="1:27" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="35"/>
       <c r="B35" s="35"/>
-      <c r="C35" s="57" t="s">
+      <c r="C35" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="D35" s="57"/>
+      <c r="D35" s="61"/>
       <c r="E35" s="56"/>
-      <c r="F35" s="57"/>
-      <c r="G35" s="57"/>
+      <c r="F35" s="61"/>
+      <c r="G35" s="61"/>
       <c r="H35" s="44" t="s">
-        <v>14</v>
-      </c>
-      <c r="I35" s="58"/>
-      <c r="J35" s="58"/>
+        <v>13</v>
+      </c>
+      <c r="I35" s="62"/>
+      <c r="J35" s="62"/>
       <c r="P35" s="3"/>
       <c r="Q35" s="19"/>
       <c r="R35" s="28"/>
@@ -2320,7 +2320,7 @@
     </row>
     <row r="40" spans="1:27" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="30" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B40" s="30"/>
       <c r="C40" s="30"/>
@@ -2341,27 +2341,34 @@
     </row>
     <row r="41" spans="1:27" ht="13.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="42" spans="1:27" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="59" t="s">
-        <v>13</v>
-      </c>
-      <c r="B42" s="59"/>
-      <c r="C42" s="59"/>
-      <c r="D42" s="59"/>
-      <c r="E42" s="59"/>
-      <c r="F42" s="59"/>
-      <c r="G42" s="59"/>
-      <c r="H42" s="59"/>
-      <c r="I42" s="59"/>
-      <c r="J42" s="59"/>
-      <c r="K42" s="59"/>
-      <c r="L42" s="59"/>
-      <c r="M42" s="59"/>
-      <c r="N42" s="59"/>
+      <c r="A42" s="63" t="s">
+        <v>12</v>
+      </c>
+      <c r="B42" s="63"/>
+      <c r="C42" s="63"/>
+      <c r="D42" s="63"/>
+      <c r="E42" s="63"/>
+      <c r="F42" s="63"/>
+      <c r="G42" s="63"/>
+      <c r="H42" s="63"/>
+      <c r="I42" s="63"/>
+      <c r="J42" s="63"/>
+      <c r="K42" s="63"/>
+      <c r="L42" s="63"/>
+      <c r="M42" s="63"/>
+      <c r="N42" s="63"/>
     </row>
     <row r="43" spans="1:27" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="44" spans="1:27" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="A42:N42"/>
+    <mergeCell ref="S11:T11"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A13:N13"/>
     <mergeCell ref="A7:N7"/>
     <mergeCell ref="A8:N8"/>
     <mergeCell ref="W33:X33"/>
@@ -2369,13 +2376,6 @@
     <mergeCell ref="X8:Y8"/>
     <mergeCell ref="V9:W9"/>
     <mergeCell ref="X9:Y9"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="A42:N42"/>
-    <mergeCell ref="S11:T11"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="A13:N13"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.59055118110236227" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>

<commit_message>
fix: resync production excel templates
</commit_message>
<xml_diff>
--- a/app/templates/Template_Compresion.xlsx
+++ b/app/templates/Template_Compresion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448594CE-AF0B-4DD2-9B69-10FFD032C8E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7B7706-5A5F-41F4-B7FE-463F37FB4391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7452" yWindow="1788" windowWidth="16284" windowHeight="9828" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="92" r:id="rId1"/>
@@ -1152,28 +1152,28 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>779288</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>75275</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>580846</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>200976</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>141950</xdr:rowOff>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Imagen 10">
+        <xdr:cNvPr id="7" name="Imagen 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{24E688ED-D05A-43BC-986F-7FC9B0118FBB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93516DB8-BCC6-4A83-A8D2-E189424AE1DE}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1184,29 +1184,18 @@
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="2684288" y="75275"/>
-          <a:ext cx="1344954" cy="759402"/>
+          <a:off x="3429000" y="0"/>
+          <a:ext cx="1435416" cy="845820"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>

</xml_diff>

<commit_message>
feat: agregar nombre_equipo en esquema y Excel, template actualizado con columna fecha_revisado
</commit_message>
<xml_diff>
--- a/app/templates/Template_Compresion.xlsx
+++ b/app/templates/Template_Compresion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7B7706-5A5F-41F4-B7FE-463F37FB4391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D7DDB41-7C0E-4A25-BA0E-E4FE2898A1DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="FORMATO" sheetId="92" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">FORMATO!$A$1:$N$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">FORMATO!$A$1:$O$42</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>LABORATORIO DE ENSAYO DE MATERIALES</t>
   </si>
@@ -102,7 +102,7 @@
     <t>Realizado</t>
   </si>
   <si>
-    <t>Versión: 04 (23-03-2026)</t>
+    <t>Versión: 04 (17-02-2026)</t>
   </si>
 </sst>
 </file>
@@ -796,7 +796,7 @@
       <xdr:rowOff>121920</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>74264</xdr:colOff>
       <xdr:row>40</xdr:row>
       <xdr:rowOff>121920</xdr:rowOff>
@@ -1554,7 +1554,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:AA44"/>
+  <dimension ref="A1:AB44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="1.33203125" style="1" customWidth="1"/>
@@ -1565,21 +1565,21 @@
     <col min="7" max="7" width="11.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="11.33203125" style="1" customWidth="1"/>
     <col min="9" max="9" width="10.33203125" style="1" customWidth="1"/>
-    <col min="10" max="13" width="9.109375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="1.109375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="6.44140625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="4.109375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="8" style="1" customWidth="1"/>
-    <col min="18" max="18" width="10.33203125" style="1"/>
-    <col min="19" max="19" width="2.6640625" style="1" customWidth="1"/>
-    <col min="20" max="21" width="10.33203125" style="1"/>
-    <col min="22" max="22" width="16.88671875" style="1" customWidth="1"/>
-    <col min="23" max="24" width="10.33203125" style="1"/>
-    <col min="25" max="27" width="5.6640625" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="10.33203125" style="1"/>
+    <col min="10" max="14" width="9.109375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="1.109375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="6.44140625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.109375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="8" style="1" customWidth="1"/>
+    <col min="19" max="19" width="10.33203125" style="1"/>
+    <col min="20" max="20" width="2.6640625" style="1" customWidth="1"/>
+    <col min="21" max="22" width="10.33203125" style="1"/>
+    <col min="23" max="23" width="16.88671875" style="1" customWidth="1"/>
+    <col min="24" max="25" width="10.33203125" style="1"/>
+    <col min="26" max="28" width="5.6640625" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="10.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" ht="14.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A1" s="32"/>
       <c r="B1" s="45"/>
       <c r="C1" s="8"/>
@@ -1593,9 +1593,10 @@
       <c r="K1" s="9"/>
       <c r="L1" s="9"/>
       <c r="M1" s="9"/>
-      <c r="N1" s="10"/>
-    </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N1" s="9"/>
+      <c r="O1" s="10"/>
+    </row>
+    <row r="2" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="33"/>
       <c r="C2" s="5"/>
       <c r="D2" s="6"/>
@@ -1608,9 +1609,10 @@
       <c r="K2" s="6"/>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
-      <c r="N2" s="11"/>
-    </row>
-    <row r="3" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N2" s="6"/>
+      <c r="O2" s="11"/>
+    </row>
+    <row r="3" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="33"/>
       <c r="C3" s="5"/>
       <c r="D3" s="6"/>
@@ -1623,9 +1625,10 @@
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="11"/>
-    </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N3" s="6"/>
+      <c r="O3" s="11"/>
+    </row>
+    <row r="4" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="33"/>
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
@@ -1638,9 +1641,10 @@
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
       <c r="M4" s="6"/>
-      <c r="N4" s="11"/>
-    </row>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N4" s="6"/>
+      <c r="O4" s="11"/>
+    </row>
+    <row r="5" spans="1:27" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="34"/>
       <c r="B5" s="46"/>
       <c r="C5" s="7"/>
@@ -1654,9 +1658,10 @@
       <c r="K5" s="7"/>
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
-      <c r="N5" s="12"/>
-    </row>
-    <row r="6" spans="1:26" ht="6.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="N5" s="7"/>
+      <c r="O5" s="12"/>
+    </row>
+    <row r="6" spans="1:27" ht="6.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
@@ -1669,8 +1674,9 @@
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
       <c r="N6" s="4"/>
-    </row>
-    <row r="7" spans="1:26" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O6" s="4"/>
+    </row>
+    <row r="7" spans="1:27" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="57" t="s">
         <v>0</v>
       </c>
@@ -1687,8 +1693,9 @@
       <c r="L7" s="57"/>
       <c r="M7" s="57"/>
       <c r="N7" s="57"/>
-    </row>
-    <row r="8" spans="1:26" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O7" s="57"/>
+    </row>
+    <row r="8" spans="1:27" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="58" t="s">
         <v>1</v>
       </c>
@@ -1705,13 +1712,14 @@
       <c r="L8" s="58"/>
       <c r="M8" s="58"/>
       <c r="N8" s="58"/>
-      <c r="V8" s="60"/>
+      <c r="O8" s="58"/>
       <c r="W8" s="60"/>
       <c r="X8" s="60"/>
       <c r="Y8" s="60"/>
-      <c r="Z8" s="15"/>
-    </row>
-    <row r="9" spans="1:26" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z8" s="60"/>
+      <c r="AA8" s="15"/>
+    </row>
+    <row r="9" spans="1:27" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
@@ -1724,19 +1732,20 @@
       <c r="L9" s="13"/>
       <c r="M9" s="13"/>
       <c r="N9" s="13"/>
-      <c r="V9" s="60"/>
+      <c r="O9" s="13"/>
       <c r="W9" s="60"/>
       <c r="X9" s="60"/>
       <c r="Y9" s="60"/>
-      <c r="Z9" s="15"/>
-    </row>
-    <row r="10" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Z9" s="60"/>
+      <c r="AA9" s="15"/>
+    </row>
+    <row r="10" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="14"/>
-      <c r="N10" s="13"/>
-      <c r="P10" s="3"/>
+      <c r="O10" s="13"/>
       <c r="Q10" s="3"/>
-    </row>
-    <row r="11" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R10" s="3"/>
+    </row>
+    <row r="11" spans="1:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="14"/>
       <c r="D11" s="29"/>
       <c r="E11" s="29"/>
@@ -1748,13 +1757,14 @@
       <c r="K11" s="29"/>
       <c r="L11" s="29"/>
       <c r="M11" s="29"/>
-      <c r="N11" s="13"/>
-      <c r="P11" s="3"/>
+      <c r="N11" s="29"/>
+      <c r="O11" s="13"/>
       <c r="Q11" s="3"/>
-      <c r="S11" s="64"/>
+      <c r="R11" s="3"/>
       <c r="T11" s="64"/>
-    </row>
-    <row r="12" spans="1:26" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U11" s="64"/>
+    </row>
+    <row r="12" spans="1:27" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="65" t="s">
         <v>2</v>
       </c>
@@ -1770,12 +1780,13 @@
       <c r="K12" s="66"/>
       <c r="L12" s="66"/>
       <c r="M12" s="66"/>
-      <c r="N12" s="67"/>
-      <c r="O12" s="3"/>
+      <c r="N12" s="66"/>
+      <c r="O12" s="67"/>
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
-    </row>
-    <row r="13" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R12" s="3"/>
+    </row>
+    <row r="13" spans="1:27" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="68" t="s">
         <v>3</v>
       </c>
@@ -1791,16 +1802,17 @@
       <c r="K13" s="69"/>
       <c r="L13" s="69"/>
       <c r="M13" s="69"/>
-      <c r="N13" s="70"/>
-      <c r="O13" s="3"/>
+      <c r="N13" s="69"/>
+      <c r="O13" s="70"/>
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
-    </row>
-    <row r="14" spans="1:26" ht="7.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O14" s="3"/>
+      <c r="R13" s="3"/>
+    </row>
+    <row r="14" spans="1:27" ht="7.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="P14" s="3"/>
-    </row>
-    <row r="15" spans="1:26" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q14" s="3"/>
+    </row>
+    <row r="15" spans="1:27" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="41" t="s">
         <v>14</v>
       </c>
@@ -1832,13 +1844,16 @@
         <v>16</v>
       </c>
       <c r="L15" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="M15" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="M15" s="43" t="s">
+      <c r="N15" s="43" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="50">
         <v>1</v>
       </c>
@@ -1851,10 +1866,11 @@
       <c r="I16" s="49"/>
       <c r="J16" s="49"/>
       <c r="K16" s="55"/>
-      <c r="L16" s="49"/>
-      <c r="M16" s="55"/>
-    </row>
-    <row r="17" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L16" s="55"/>
+      <c r="M16" s="49"/>
+      <c r="N16" s="55"/>
+    </row>
+    <row r="17" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="50">
         <v>2</v>
       </c>
@@ -1869,8 +1885,9 @@
       <c r="K17" s="50"/>
       <c r="L17" s="50"/>
       <c r="M17" s="50"/>
-    </row>
-    <row r="18" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N17" s="50"/>
+    </row>
+    <row r="18" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="50">
         <v>3</v>
       </c>
@@ -1885,10 +1902,11 @@
       <c r="K18" s="50"/>
       <c r="L18" s="50"/>
       <c r="M18" s="50"/>
-      <c r="O18" s="3"/>
+      <c r="N18" s="50"/>
       <c r="P18" s="3"/>
-    </row>
-    <row r="19" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q18" s="3"/>
+    </row>
+    <row r="19" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="50">
         <v>4</v>
       </c>
@@ -1903,11 +1921,12 @@
       <c r="K19" s="53"/>
       <c r="L19" s="53"/>
       <c r="M19" s="53"/>
-      <c r="N19" s="16"/>
-      <c r="O19" s="3"/>
+      <c r="N19" s="53"/>
+      <c r="O19" s="16"/>
       <c r="P19" s="3"/>
-    </row>
-    <row r="20" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q19" s="3"/>
+    </row>
+    <row r="20" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="50">
         <v>5</v>
       </c>
@@ -1922,11 +1941,12 @@
       <c r="K20" s="53"/>
       <c r="L20" s="53"/>
       <c r="M20" s="53"/>
-      <c r="N20" s="16"/>
-      <c r="O20" s="3"/>
+      <c r="N20" s="53"/>
+      <c r="O20" s="16"/>
       <c r="P20" s="3"/>
-    </row>
-    <row r="21" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q20" s="3"/>
+    </row>
+    <row r="21" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="50">
         <v>6</v>
       </c>
@@ -1941,11 +1961,12 @@
       <c r="K21" s="53"/>
       <c r="L21" s="53"/>
       <c r="M21" s="53"/>
-      <c r="N21" s="16"/>
-      <c r="O21" s="3"/>
+      <c r="N21" s="53"/>
+      <c r="O21" s="16"/>
       <c r="P21" s="3"/>
-    </row>
-    <row r="22" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q21" s="3"/>
+    </row>
+    <row r="22" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="50">
         <v>7</v>
       </c>
@@ -1960,11 +1981,12 @@
       <c r="K22" s="53"/>
       <c r="L22" s="53"/>
       <c r="M22" s="53"/>
-      <c r="N22" s="16"/>
-      <c r="O22" s="3"/>
+      <c r="N22" s="53"/>
+      <c r="O22" s="16"/>
       <c r="P22" s="3"/>
-    </row>
-    <row r="23" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q22" s="3"/>
+    </row>
+    <row r="23" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="50">
         <v>8</v>
       </c>
@@ -1979,11 +2001,12 @@
       <c r="K23" s="53"/>
       <c r="L23" s="53"/>
       <c r="M23" s="53"/>
-      <c r="N23" s="16"/>
-      <c r="O23" s="3"/>
+      <c r="N23" s="53"/>
+      <c r="O23" s="16"/>
       <c r="P23" s="3"/>
-    </row>
-    <row r="24" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q23" s="3"/>
+    </row>
+    <row r="24" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="50">
         <v>9</v>
       </c>
@@ -1998,11 +2021,12 @@
       <c r="K24" s="53"/>
       <c r="L24" s="53"/>
       <c r="M24" s="53"/>
-      <c r="N24" s="16"/>
-      <c r="O24" s="3"/>
+      <c r="N24" s="53"/>
+      <c r="O24" s="16"/>
       <c r="P24" s="3"/>
-    </row>
-    <row r="25" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q24" s="3"/>
+    </row>
+    <row r="25" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="50">
         <v>10</v>
       </c>
@@ -2017,11 +2041,12 @@
       <c r="K25" s="53"/>
       <c r="L25" s="53"/>
       <c r="M25" s="53"/>
-      <c r="N25" s="16"/>
-      <c r="O25" s="3"/>
+      <c r="N25" s="53"/>
+      <c r="O25" s="16"/>
       <c r="P25" s="3"/>
-    </row>
-    <row r="26" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q25" s="3"/>
+    </row>
+    <row r="26" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="50">
         <v>11</v>
       </c>
@@ -2036,11 +2061,12 @@
       <c r="K26" s="53"/>
       <c r="L26" s="53"/>
       <c r="M26" s="53"/>
-      <c r="N26" s="16"/>
-      <c r="O26" s="3"/>
+      <c r="N26" s="53"/>
+      <c r="O26" s="16"/>
       <c r="P26" s="3"/>
-    </row>
-    <row r="27" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q26" s="3"/>
+    </row>
+    <row r="27" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="50">
         <v>12</v>
       </c>
@@ -2055,11 +2081,12 @@
       <c r="K27" s="53"/>
       <c r="L27" s="53"/>
       <c r="M27" s="53"/>
-      <c r="N27" s="16"/>
-      <c r="O27" s="3"/>
+      <c r="N27" s="53"/>
+      <c r="O27" s="16"/>
       <c r="P27" s="3"/>
-    </row>
-    <row r="28" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q27" s="3"/>
+    </row>
+    <row r="28" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="50">
         <v>13</v>
       </c>
@@ -2074,11 +2101,12 @@
       <c r="K28" s="53"/>
       <c r="L28" s="53"/>
       <c r="M28" s="53"/>
-      <c r="N28" s="16"/>
-      <c r="O28" s="3"/>
+      <c r="N28" s="53"/>
+      <c r="O28" s="16"/>
       <c r="P28" s="3"/>
-    </row>
-    <row r="29" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q28" s="3"/>
+    </row>
+    <row r="29" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="50">
         <v>14</v>
       </c>
@@ -2093,11 +2121,12 @@
       <c r="K29" s="53"/>
       <c r="L29" s="53"/>
       <c r="M29" s="53"/>
-      <c r="N29" s="16"/>
-      <c r="O29" s="3"/>
+      <c r="N29" s="53"/>
+      <c r="O29" s="16"/>
       <c r="P29" s="3"/>
-    </row>
-    <row r="30" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q29" s="3"/>
+    </row>
+    <row r="30" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="50">
         <v>15</v>
       </c>
@@ -2112,11 +2141,12 @@
       <c r="K30" s="53"/>
       <c r="L30" s="53"/>
       <c r="M30" s="53"/>
-      <c r="N30" s="16"/>
-      <c r="O30" s="3"/>
+      <c r="N30" s="53"/>
+      <c r="O30" s="16"/>
       <c r="P30" s="3"/>
-    </row>
-    <row r="31" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q30" s="3"/>
+    </row>
+    <row r="31" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="50">
         <v>16</v>
       </c>
@@ -2131,11 +2161,12 @@
       <c r="K31" s="53"/>
       <c r="L31" s="53"/>
       <c r="M31" s="53"/>
-      <c r="N31" s="16"/>
-      <c r="O31" s="3"/>
+      <c r="N31" s="53"/>
+      <c r="O31" s="16"/>
       <c r="P31" s="3"/>
-    </row>
-    <row r="32" spans="2:16" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q31" s="3"/>
+    </row>
+    <row r="32" spans="2:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="50">
         <v>17</v>
       </c>
@@ -2150,11 +2181,12 @@
       <c r="K32" s="53"/>
       <c r="L32" s="53"/>
       <c r="M32" s="53"/>
-      <c r="N32" s="16"/>
-      <c r="O32" s="3"/>
+      <c r="N32" s="53"/>
+      <c r="O32" s="16"/>
       <c r="P32" s="3"/>
-    </row>
-    <row r="33" spans="1:27" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q32" s="3"/>
+    </row>
+    <row r="33" spans="1:28" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="36"/>
       <c r="B33" s="50">
         <v>18</v>
@@ -2170,19 +2202,20 @@
       <c r="K33" s="53"/>
       <c r="L33" s="53"/>
       <c r="M33" s="53"/>
-      <c r="N33" s="36"/>
-      <c r="O33" s="20"/>
-      <c r="P33" s="17"/>
-      <c r="Q33" s="19"/>
-      <c r="R33" s="4"/>
+      <c r="N33" s="53"/>
+      <c r="O33" s="36"/>
+      <c r="P33" s="20"/>
+      <c r="Q33" s="17"/>
+      <c r="R33" s="19"/>
       <c r="S33" s="4"/>
-      <c r="T33" s="20"/>
+      <c r="T33" s="4"/>
       <c r="U33" s="20"/>
       <c r="V33" s="20"/>
-      <c r="W33" s="59"/>
+      <c r="W33" s="20"/>
       <c r="X33" s="59"/>
-    </row>
-    <row r="34" spans="1:27" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y33" s="59"/>
+    </row>
+    <row r="34" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="35"/>
       <c r="B34" s="35"/>
       <c r="C34" s="35"/>
@@ -2197,15 +2230,16 @@
       <c r="L34" s="35"/>
       <c r="M34" s="35"/>
       <c r="N34" s="35"/>
-      <c r="O34" s="20"/>
-      <c r="P34" s="17"/>
-      <c r="Q34" s="19"/>
-      <c r="R34" s="20"/>
-      <c r="T34" s="23"/>
-      <c r="V34" s="25"/>
-      <c r="W34" s="24"/>
-    </row>
-    <row r="35" spans="1:27" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O34" s="35"/>
+      <c r="P34" s="20"/>
+      <c r="Q34" s="17"/>
+      <c r="R34" s="19"/>
+      <c r="S34" s="20"/>
+      <c r="U34" s="23"/>
+      <c r="W34" s="25"/>
+      <c r="X34" s="24"/>
+    </row>
+    <row r="35" spans="1:28" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="35"/>
       <c r="B35" s="35"/>
       <c r="C35" s="61" t="s">
@@ -2220,34 +2254,34 @@
       </c>
       <c r="I35" s="62"/>
       <c r="J35" s="62"/>
-      <c r="P35" s="3"/>
-      <c r="Q35" s="19"/>
-      <c r="R35" s="28"/>
-      <c r="T35" s="26"/>
-      <c r="U35" s="23"/>
-      <c r="V35" s="21"/>
+      <c r="Q35" s="3"/>
+      <c r="R35" s="19"/>
+      <c r="S35" s="28"/>
+      <c r="U35" s="26"/>
+      <c r="V35" s="23"/>
       <c r="W35" s="21"/>
       <c r="X35" s="21"/>
-      <c r="Y35" s="22"/>
-      <c r="Z35" s="27"/>
-      <c r="AA35" s="22"/>
-    </row>
-    <row r="36" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y35" s="21"/>
+      <c r="Z35" s="22"/>
+      <c r="AA35" s="27"/>
+      <c r="AB35" s="22"/>
+    </row>
+    <row r="36" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="39"/>
       <c r="B36" s="39"/>
-      <c r="P36" s="3"/>
-      <c r="Q36" s="19"/>
-      <c r="R36" s="28"/>
-      <c r="T36" s="26"/>
-      <c r="U36" s="23"/>
-      <c r="V36" s="21"/>
+      <c r="Q36" s="3"/>
+      <c r="R36" s="19"/>
+      <c r="S36" s="28"/>
+      <c r="U36" s="26"/>
+      <c r="V36" s="23"/>
       <c r="W36" s="21"/>
       <c r="X36" s="21"/>
-      <c r="Y36" s="22"/>
-      <c r="Z36" s="27"/>
-      <c r="AA36" s="22"/>
-    </row>
-    <row r="37" spans="1:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y36" s="21"/>
+      <c r="Z36" s="22"/>
+      <c r="AA36" s="27"/>
+      <c r="AB36" s="22"/>
+    </row>
+    <row r="37" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="38" t="s">
         <v>10</v>
       </c>
@@ -2263,19 +2297,20 @@
       <c r="K37" s="37"/>
       <c r="L37" s="37"/>
       <c r="M37" s="37"/>
-      <c r="P37" s="3"/>
-      <c r="Q37" s="19"/>
-      <c r="R37" s="28"/>
-      <c r="T37" s="26"/>
-      <c r="U37" s="23"/>
-      <c r="V37" s="21"/>
+      <c r="N37" s="37"/>
+      <c r="Q37" s="3"/>
+      <c r="R37" s="19"/>
+      <c r="S37" s="28"/>
+      <c r="U37" s="26"/>
+      <c r="V37" s="23"/>
       <c r="W37" s="21"/>
       <c r="X37" s="21"/>
-      <c r="Y37" s="22"/>
-      <c r="Z37" s="27"/>
-      <c r="AA37" s="22"/>
-    </row>
-    <row r="38" spans="1:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y37" s="21"/>
+      <c r="Z37" s="22"/>
+      <c r="AA37" s="27"/>
+      <c r="AB37" s="22"/>
+    </row>
+    <row r="38" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D38" s="31"/>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -2286,28 +2321,29 @@
       <c r="K38" s="31"/>
       <c r="L38" s="31"/>
       <c r="M38" s="31"/>
-      <c r="P38" s="3"/>
-      <c r="Q38" s="18"/>
-      <c r="R38" s="28"/>
-      <c r="T38" s="26"/>
-      <c r="U38" s="23"/>
-      <c r="V38" s="21"/>
+      <c r="N38" s="31"/>
+      <c r="Q38" s="3"/>
+      <c r="R38" s="18"/>
+      <c r="S38" s="28"/>
+      <c r="U38" s="26"/>
+      <c r="V38" s="23"/>
       <c r="W38" s="21"/>
       <c r="X38" s="21"/>
-      <c r="Y38" s="22"/>
-      <c r="Z38" s="27"/>
-      <c r="AA38" s="22"/>
-    </row>
-    <row r="39" spans="1:27" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y38" s="21"/>
+      <c r="Z38" s="22"/>
+      <c r="AA38" s="27"/>
+      <c r="AB38" s="22"/>
+    </row>
+    <row r="39" spans="1:28" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="30" t="s">
         <v>11</v>
       </c>
       <c r="B39" s="30"/>
       <c r="C39" s="30"/>
-      <c r="O39" s="21"/>
-      <c r="P39" s="3"/>
-    </row>
-    <row r="40" spans="1:27" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P39" s="21"/>
+      <c r="Q39" s="3"/>
+    </row>
+    <row r="40" spans="1:28" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="30" t="s">
         <v>21</v>
       </c>
@@ -2324,12 +2360,13 @@
       <c r="L40" s="2"/>
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
-      <c r="O40" s="3"/>
+      <c r="O40" s="2"/>
       <c r="P40" s="3"/>
       <c r="Q40" s="3"/>
-    </row>
-    <row r="41" spans="1:27" ht="13.95" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:27" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R40" s="3"/>
+    </row>
+    <row r="41" spans="1:28" ht="13.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:28" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="63" t="s">
         <v>12</v>
       </c>
@@ -2346,25 +2383,26 @@
       <c r="L42" s="63"/>
       <c r="M42" s="63"/>
       <c r="N42" s="63"/>
-    </row>
-    <row r="43" spans="1:27" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:27" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="O42" s="63"/>
+    </row>
+    <row r="43" spans="1:28" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:28" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="F35:G35"/>
     <mergeCell ref="I35:J35"/>
-    <mergeCell ref="A42:N42"/>
-    <mergeCell ref="S11:T11"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="A13:N13"/>
-    <mergeCell ref="A7:N7"/>
-    <mergeCell ref="A8:N8"/>
-    <mergeCell ref="W33:X33"/>
-    <mergeCell ref="V8:W8"/>
-    <mergeCell ref="X8:Y8"/>
-    <mergeCell ref="V9:W9"/>
-    <mergeCell ref="X9:Y9"/>
+    <mergeCell ref="A42:O42"/>
+    <mergeCell ref="T11:U11"/>
+    <mergeCell ref="A12:O12"/>
+    <mergeCell ref="A13:O13"/>
+    <mergeCell ref="A7:O7"/>
+    <mergeCell ref="A8:O8"/>
+    <mergeCell ref="X33:Y33"/>
+    <mergeCell ref="W8:X8"/>
+    <mergeCell ref="Y8:Z8"/>
+    <mergeCell ref="W9:X9"/>
+    <mergeCell ref="Y9:Z9"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.59055118110236227" bottom="0.39370078740157483" header="0" footer="0"/>

</xml_diff>

<commit_message>
fix: eliminar absPath de workbook.xml que causaba advertencia de vínculos en Excel
</commit_message>
<xml_diff>
--- a/app/templates/Template_Compresion.xlsx
+++ b/app/templates/Template_Compresion.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D7DDB41-7C0E-4A25-BA0E-E4FE2898A1DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>

</xml_diff>